<commit_message>
Add final ADSS app
</commit_message>
<xml_diff>
--- a/artifacts/evaluation_suite/contract_nli/contract_nli_paper_tables.xlsx
+++ b/artifacts/evaluation_suite/contract_nli/contract_nli_paper_tables.xlsx
@@ -12,12 +12,14 @@
     <sheet name="Raw_Main" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Table3_Ablation" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Raw_Ablation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Table5_Strict" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Table5_Uncertainty" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Table6_ErrorProps" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Error_Cases" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="McNemar" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Diagnostics_Strict" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Table4_Contestability" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Table5_Strict" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Table5_Uncertainty" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Robustness" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Table6_ErrorProps" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Error_Cases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="McNemar" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Diagnostics_Strict" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -573,15 +575,723 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>proportion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>argument_omission</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.67</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>83.33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>strength_miscalibration</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>alternative_claim_alignment_error</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>threshold_uncertainty_failure</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>task_transfer_failure</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>gold_label</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>predicted_label</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sigma_phi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>test_0003</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.4974999999999999</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>test_0007</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.400375</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test_0009</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1.898437499980865e-06</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>test_0010</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7.499999999999174e-05</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>test_0011</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.40000421875</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>test_0012</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5.625000000009095e-06</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>test_0013</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>argument_omission</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>No relevant arguments were retained for the target claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>test_0014</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.4320937499999999</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>test_0015</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.404425</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>test_0016</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.37500003125</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>test_0020</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.45008</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>test_0021</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>argument_omission</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>No relevant arguments were retained for the target claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>test_0026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.009499999999999899</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>test_0027</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.0002249999999999</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>test_0033</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.4708</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>test_0038</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>argument_omission</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No relevant arguments were retained for the target claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>test_0039</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>UNCERTAIN</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.50425</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>test_0062</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.56625</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>relation_error</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -624,19 +1334,67 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADSS w/o Symbolic Solver</t>
+          <t>Zero-shot CoT</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>5</v>
       </c>
       <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Full ADSS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Few-shot Prompting</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.454545454545455</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2265625</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Full ADSS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADSS w/o Symbolic Solver</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
         <v>1.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F4" t="n">
         <v>0.21875</v>
       </c>
     </row>
@@ -645,7 +1403,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5461,7 +6219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5585,122 +6343,244 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADSS w/o Symbolic Solver</t>
+          <t>Zero-shot CoT</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>82</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7317</v>
+        <v>0.7683</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7147</v>
+        <v>0.7551</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0732</v>
+        <v>0.2317</v>
       </c>
       <c r="G2" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9077</v>
+        <v>0.7683</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8991</v>
+        <v>0.7551</v>
       </c>
       <c r="J2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0588</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0556</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>73.17</v>
+        <v>76.83</v>
       </c>
       <c r="N2" t="n">
-        <v>71.47</v>
+        <v>75.51000000000001</v>
       </c>
       <c r="O2" t="n">
-        <v>7.32</v>
+        <v>23.17</v>
       </c>
       <c r="P2" t="n">
-        <v>90.77</v>
+        <v>76.83</v>
       </c>
       <c r="Q2" t="n">
-        <v>89.91</v>
+        <v>75.51000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>5.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Full ADSS</t>
+          <t>Few-shot Prompting</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>82</v>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8415</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.8374</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1585</v>
+      </c>
+      <c r="G3" t="n">
+        <v>82</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8415</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.8374</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="N3" t="n">
+        <v>83.73999999999999</v>
+      </c>
+      <c r="O3" t="n">
+        <v>15.85</v>
+      </c>
+      <c r="P3" t="n">
+        <v>84.15000000000001</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>83.73999999999999</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADSS w/o Symbolic Solver</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>82</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.7317</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7147</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0732</v>
+      </c>
+      <c r="G4" t="n">
+        <v>65</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9077</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.8991</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0588</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0556</v>
+      </c>
+      <c r="M4" t="n">
+        <v>73.17</v>
+      </c>
+      <c r="N4" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="O4" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="P4" t="n">
+        <v>90.77</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>89.91</v>
+      </c>
+      <c r="R4" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="S4" t="n">
+        <v>5.56</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full ADSS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>82</v>
+      </c>
+      <c r="C5" t="n">
         <v>8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D5" t="n">
         <v>0.7805</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E5" t="n">
         <v>0.7718</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F5" t="n">
         <v>0.1341</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G5" t="n">
         <v>74</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H5" t="n">
         <v>0.8514</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I5" t="n">
         <v>0.845</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J5" t="n">
         <v>8</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K5" t="n">
         <v>0.125</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L5" t="n">
         <v>0.1111</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M5" t="n">
         <v>78.05</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N5" t="n">
         <v>77.18000000000001</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O5" t="n">
         <v>13.41</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P5" t="n">
         <v>85.14</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q5" t="n">
         <v>84.5</v>
       </c>
-      <c r="R3" t="n">
+      <c r="R5" t="n">
         <v>12.5</v>
       </c>
-      <c r="S3" t="n">
+      <c r="S5" t="n">
         <v>11.11</v>
       </c>
     </row>
@@ -5715,7 +6595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5821,104 +6701,208 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADSS w/o Symbolic Solver</t>
+          <t>Zero-shot CoT</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>82</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7317073170731707</v>
+        <v>0.7682926829268293</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6341463414634146</v>
+        <v>0.6707317073170732</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8292682926829268</v>
+        <v>0.8658536585365854</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7147375079063883</v>
+        <v>0.7551469432657552</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6095238095238096</v>
+        <v>0.6620879120879122</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8123569794050344</v>
+        <v>0.8444022770398482</v>
       </c>
       <c r="J2" t="n">
-        <v>0.073170731707317</v>
+        <v>0.2317073170731707</v>
       </c>
       <c r="K2" t="n">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9076923076923076</v>
+        <v>0.7682926829268293</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8990683229813664</v>
+        <v>0.7551469432657552</v>
       </c>
       <c r="N2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0588235294117647</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0555555555555555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Full ADSS</t>
+          <t>Few-shot Prompting</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>82</v>
       </c>
       <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8414634146341463</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.7560975609756098</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9146341463414634</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.8373760488176965</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.7485068603712672</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.9145197319434102</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.1585365853658536</v>
+      </c>
+      <c r="K3" t="n">
+        <v>82</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8414634146341463</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.8373760488176965</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADSS w/o Symbolic Solver</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>82</v>
+      </c>
+      <c r="C4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.7317073170731707</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6341463414634146</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.8292682926829268</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.7147375079063883</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.6095238095238096</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.8123569794050344</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.073170731707317</v>
+      </c>
+      <c r="K4" t="n">
+        <v>65</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9076923076923076</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.8990683229813664</v>
+      </c>
+      <c r="N4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.0588235294117647</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0555555555555555</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full ADSS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>82</v>
+      </c>
+      <c r="C5" t="n">
         <v>8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D5" t="n">
         <v>0.7804878048780488</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E5" t="n">
         <v>0.6829268292682927</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F5" t="n">
         <v>0.8658536585365854</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G5" t="n">
         <v>0.771799628942486</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H5" t="n">
         <v>0.6778249253496778</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I5" t="n">
         <v>0.8536585365853659</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J5" t="n">
         <v>0.1341463414634146</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K5" t="n">
         <v>74</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L5" t="n">
         <v>0.8513513513513513</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M5" t="n">
         <v>0.8449819082079604</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N5" t="n">
         <v>8</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O5" t="n">
         <v>0.125</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P5" t="n">
         <v>0.1111111111111111</v>
       </c>
     </row>
@@ -6533,6 +7517,128 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>regime</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_total</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>decision_flip_rate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>corrective_flip_rate</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>minimal_edit_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>score_shift_magnitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>decision_flip_rate_%</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>corrective_flip_rate_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>oracle</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>82</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1829</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.1829</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.066666666666667</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1479</v>
+      </c>
+      <c r="G2" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="H2" t="n">
+        <v>18.29</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>82</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.09760000000000001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0366</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0546</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6815,7 +7921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6973,707 +8079,383 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>proportion</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>percentage</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>argument_omission</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="C2" t="n">
-        <v>16.67</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="C3" t="n">
-        <v>83.33</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>strength_miscalibration</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>alternative_claim_alignment_error</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>threshold_uncertainty_failure</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>task_transfer_failure</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>case_id</t>
+          <t>perturbation</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>gold_label</t>
+          <t>p</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>predicted_label</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sigma_phi</t>
+          <t>score_stability_delta_p</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>accuracy</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>reason</t>
+          <t>macro_f1</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test_0003</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
+          <t>argument_removal</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>82</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4974999999999999</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test_0007</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>argument_removal</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>82</v>
       </c>
       <c r="D3" t="n">
-        <v>0.400375</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test_0009</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>argument_removal</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>82</v>
       </c>
       <c r="D4" t="n">
-        <v>1.898437499980865e-06</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.0326</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test_0010</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>argument_removal</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>82</v>
       </c>
       <c r="D5" t="n">
-        <v>7.499999999999174e-05</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.0336</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.8415</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.8374</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>test_0011</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>argument_removal</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>82</v>
       </c>
       <c r="D6" t="n">
-        <v>0.40000421875</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.08890000000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7561</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.7438</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>test_0012</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>relation_flip</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>82</v>
       </c>
       <c r="D7" t="n">
-        <v>5.625000000009095e-06</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>test_0013</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
+          <t>relation_flip</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>82</v>
       </c>
       <c r="D8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>argument_omission</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>No relevant arguments were retained for the target claim.</t>
-        </is>
+        <v>0.0654</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.7439</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.7294</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>test_0014</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>relation_flip</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>82</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4320937499999999</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.2839</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.6463</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.6032999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>test_0015</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>relation_flip</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>82</v>
       </c>
       <c r="D10" t="n">
-        <v>0.404425</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.3183</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.622</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.5832000000000001</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>test_0016</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>relation_flip</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>82</v>
       </c>
       <c r="D11" t="n">
-        <v>0.37500003125</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.3555</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.4488</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>test_0020</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
+          <t>tau_noise</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>82</v>
       </c>
       <c r="D12" t="n">
-        <v>0.45008</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>test_0021</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
+          <t>tau_noise</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>82</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>argument_omission</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>No relevant arguments were retained for the target claim.</t>
-        </is>
+        <v>0.0022</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>test_0026</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>tau_noise</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>82</v>
       </c>
       <c r="D14" t="n">
-        <v>0.009499999999999899</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.0025</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.7927</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.7834</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>test_0027</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+          <t>tau_noise</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>82</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0002249999999999</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.0032</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.7805</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.7718</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>test_0033</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
+          <t>tau_noise</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>82</v>
       </c>
       <c r="D16" t="n">
-        <v>0.4708</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>test_0038</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>argument_omission</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>No relevant arguments were retained for the target claim.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>test_0039</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>UNCERTAIN</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0.50425</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>test_0062</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>0.56625</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>relation_error</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Arguments exist with non-extreme strengths; relation polarity or graph structure is the likely failure.</t>
-        </is>
+        <v>0.0068</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.7683</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.7579</v>
       </c>
     </row>
   </sheetData>

</xml_diff>